<commit_message>
Publica galeria do projeto (site/) e organiza coleções: Finais/Descartados, animacoes, avaliações
</commit_message>
<xml_diff>
--- a/Coleções/Coleção 2 - Naruto/avaliacao_colecao2.xlsx
+++ b/Coleções/Coleção 2 - Naruto/avaliacao_colecao2.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>resultado_ref1_luta_tentativa1.png</t>
+          <t>tentativa 1 - resultado_ref1_luta_tentativa1.png</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -645,23 +645,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -682,23 +670,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -711,7 +687,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>resultado_ref2_luta_tentativa1.png</t>
+          <t>tentativa 1 - resultado_ref2_luta_tentativa1.png</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -804,23 +780,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -841,23 +805,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -955,7 +907,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>resultado_ref3_luta_tentativa2.jfif</t>
+          <t>tentativa 2 - resultado_ref3_luta_tentativa2.jfif</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1048,23 +1000,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1077,7 +1017,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>resultado_ref4_luta_tentativa1.png</t>
+          <t>tentativa 1 - resultado_ref4_luta_tentativa1.png</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1170,23 +1110,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1207,23 +1135,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1236,7 +1152,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>resultado imagem 5.jpeg</t>
+          <t>tentativa 1 - resultado imagem 5.jpeg</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1264,16 +1180,11 @@
           <t>não</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
           <t>—</t>
@@ -1301,7 +1212,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>resultado imagem 5 tentativa 2.jfif</t>
+          <t>tentativa 2 - resultado imagem 5 tentativa 2.jfif</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1329,16 +1240,11 @@
           <t>não</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>—</t>
@@ -1366,7 +1272,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>tentativa 3 imagem 5.jfif</t>
+          <t>tentativa 3 - tentativa 3 imagem 5.jfif</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1394,16 +1300,11 @@
           <t>não</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>—</t>
@@ -1431,7 +1332,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>resultado imagem 6.jpeg</t>
+          <t>tentativa 1 - resultado imagem 6.jpeg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1524,23 +1425,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1561,23 +1450,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1618,16 +1495,11 @@
           <t>não</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>—</t>
@@ -1655,7 +1527,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>resultado imagem 7 tentativa 2.jfif</t>
+          <t>tentativa 2 - resultado imagem 7 tentativa 2.jfif</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1748,23 +1620,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1777,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>resultado imagem 8.jpeg</t>
+          <t>tentativa 1 - resultado imagem 8.jpeg</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1805,7 +1665,6 @@
           <t>não</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>não</t>
@@ -1826,7 +1685,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>—</t>
@@ -1854,7 +1712,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>resultado imagem 8 tentativa 2.jfif</t>
+          <t>tentativa 2 - resultado imagem 8 tentativa 2.jfif</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1882,16 +1740,11 @@
           <t>não</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>—</t>
@@ -1927,17 +1780,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>—</t>
@@ -1949,6 +1791,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Motivos de descarte em texto corrido e consistente
</commit_message>
<xml_diff>
--- a/Coleções/Coleção 2 - Naruto/avaliacao_colecao2.xlsx
+++ b/Coleções/Coleção 2 - Naruto/avaliacao_colecao2.xlsx
@@ -892,7 +892,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Descartada Q2/Q3/Q4.</t>
+          <t>Traço suavizado, sem bordas de pixel, e sombreamento diferente do original.</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Descartada C/D pose.</t>
+          <t>Pose trocada: a referência está em combate e a gerada está parada, de frente.</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Descartada C/D + mochila.</t>
+          <t>Pose trocada como na anterior, e ainda apareceu uma mochila que não existe na referência.</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Descartada C/D. Limite 3.</t>
+          <t>Pose continua estática de frente, sem corresponder ao combate da referência.</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Descartada C/D pose.</t>
+          <t>Pose de três quartos com o braço estendido, diferente da postura reta e lateral da referência.</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Descartada C/D + Q2-4.</t>
+          <t>Estrutura diferente da referência, com cores em excesso e sem bordas de pixel.</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Descartada C/D 4 poses.</t>
+          <t>Gerou quatro poses de corrida em vez de manter a pose única da referência, com detalhe inconsistente entre elas.</t>
         </is>
       </c>
     </row>

</xml_diff>